<commit_message>
Add evaluación técnico-económica OFT-128-008 Rev3
- 4_Documentos/Evaluacion_TecnicoEconomica_OFT128008_Rev3.pdf: informe
  de 7 secciones — mapeo ítems técnico/comercial, análisis crítico de
  jornadas A Demanda (474 p/días sugeridas, 0 fijas), gaps identificados
  (PEM sin estimar, precomisionado sin estimar, relocalización Shelf 6
  subestimada, seguro retroactivo May-2026) y recomendación de adjudicar
  con 3 condiciones obligatorias (caps jornadas, estimación PEM, seguro
  desde OC).
- 2_Planning/Dashboard_Inauco_Seguimiento.xlsx: nueva hoja "Eval
  Económica" con mapeo completo de ítems, tabla jornadas por actividad,
  condiciones C1-C7 y próximos pasos con fechas límite.

https://claude.ai/code/session_01ApnRXXwKuExbvPowKL5X6v
</commit_message>
<xml_diff>
--- a/2_Planning/Dashboard_Inauco_Seguimiento.xlsx
+++ b/2_Planning/Dashboard_Inauco_Seguimiento.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Portada" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="1. Hitos" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="2. Riesgos" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="3. KPIs" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="4. Dependencias" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="5. Decisiones" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="6. Entregables" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Eval Económica" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Portada" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Hitos" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. Riesgos" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. KPIs" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. Dependencias" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. Decisiones" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. Entregables" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -23,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="16">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -58,8 +59,66 @@
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="002C3E50"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001A8A3D"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="002E86C1"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00D4600A"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00B03A2E"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="18">
     <fill>
       <patternFill/>
     </fill>
@@ -91,8 +150,63 @@
         <fgColor rgb="00DBEAD5"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000D2B4E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001A5276"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001A8A3D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D5F5E3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EBF5FB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FDEBD0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FADBD8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00B03A2E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F3F4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F9E79F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -114,11 +228,25 @@
         <color rgb="00BFBFBF"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D5D8DC"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D5D8DC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D5D8DC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D5D8DC"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -141,6 +269,96 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="13" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="13" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="13" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="14" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="15" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="15" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="16" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="16" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="13" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="17" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="17" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -507,6 +725,1881 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:G68"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="11" t="inlineStr">
+        <is>
+          <t>EVALUACIÓN TÉCNICO-ECONÓMICA — OFT-128-008 Rev3</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="15" customHeight="1">
+      <c r="A2" s="12" t="inlineStr">
+        <is>
+          <t>CPF2 La Calera Fase 2 · INAUCO · Oferta Comercial 29/05/2026 · Evaluado 02/06/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="13" t="inlineStr">
+        <is>
+          <t>RECOMENDACIÓN: ADJUDICAR CON CONDICIONES (C1, C2, C3 obligatorias)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="6" customHeight="1"/>
+    <row r="5" ht="16" customHeight="1">
+      <c r="A5" s="14" t="inlineStr">
+        <is>
+          <t>1. MAPEO ÍTEMS TÉCNICOS vs. COMERCIALES</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="15" t="inlineStr">
+        <is>
+          <t>Ítem Eco.</t>
+        </is>
+      </c>
+      <c r="B6" s="15" t="inlineStr">
+        <is>
+          <t>Sistema / Descripción</t>
+        </is>
+      </c>
+      <c r="C6" s="15" t="inlineStr">
+        <is>
+          <t>Alcance Técnico Asociado</t>
+        </is>
+      </c>
+      <c r="D6" s="15" t="inlineStr">
+        <is>
+          <t>Categoría</t>
+        </is>
+      </c>
+      <c r="E6" s="15" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+      <c r="F6" s="15" t="inlineStr">
+        <is>
+          <t>Nota</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="28" customHeight="1">
+      <c r="A7" s="16" t="inlineStr">
+        <is>
+          <t>3.1.1 #1</t>
+        </is>
+      </c>
+      <c r="B7" s="17" t="inlineStr">
+        <is>
+          <t>Sist. Control Integrado CPF2-PCS-SC-07a</t>
+        </is>
+      </c>
+      <c r="C7" s="17" t="inlineStr">
+        <is>
+          <t>ControlLogix 1756, I/O HART, EN2TP PRP, MVI56E-MNETCR, Marshalling — Remota 7A (NUEVA)</t>
+        </is>
+      </c>
+      <c r="D7" s="16" t="inlineStr">
+        <is>
+          <t>Hardware+Labor</t>
+        </is>
+      </c>
+      <c r="E7" s="18" t="inlineStr">
+        <is>
+          <t>CUBIERTO</t>
+        </is>
+      </c>
+      <c r="F7" s="17" t="inlineStr">
+        <is>
+          <t>D5F5E3</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="28" customHeight="1">
+      <c r="A8" s="16" t="inlineStr">
+        <is>
+          <t>3.1.1 #2</t>
+        </is>
+      </c>
+      <c r="B8" s="17" t="inlineStr">
+        <is>
+          <t>Sist. Control Integrado CPF2-PCS-SC-07b</t>
+        </is>
+      </c>
+      <c r="C8" s="17" t="inlineStr">
+        <is>
+          <t>Ídem 07a — Remota 7B (NUEVA). Aloja controladores relocalizados desde Shelter 6</t>
+        </is>
+      </c>
+      <c r="D8" s="16" t="inlineStr">
+        <is>
+          <t>Hardware+Labor</t>
+        </is>
+      </c>
+      <c r="E8" s="18" t="inlineStr">
+        <is>
+          <t>CUBIERTO</t>
+        </is>
+      </c>
+      <c r="F8" s="17" t="inlineStr">
+        <is>
+          <t>D5F5E3</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="28" customHeight="1">
+      <c r="A9" s="16" t="inlineStr">
+        <is>
+          <t>3.1.1 #3</t>
+        </is>
+      </c>
+      <c r="B9" s="17" t="inlineStr">
+        <is>
+          <t>Sist. Comun. PMS Redundante + Skids</t>
+        </is>
+      </c>
+      <c r="C9" s="17" t="inlineStr">
+        <is>
+          <t>Switch PRP para salas ABB 800xA (Modbus TCP) + 10 paquetizados (~500 puntos)</t>
+        </is>
+      </c>
+      <c r="D9" s="16" t="inlineStr">
+        <is>
+          <t>Hardware+Labor</t>
+        </is>
+      </c>
+      <c r="E9" s="18" t="inlineStr">
+        <is>
+          <t>CUBIERTO</t>
+        </is>
+      </c>
+      <c r="F9" s="17" t="inlineStr">
+        <is>
+          <t>D5F5E3</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="28" customHeight="1">
+      <c r="A10" s="16" t="inlineStr">
+        <is>
+          <t>3.1.1 #4</t>
+        </is>
+      </c>
+      <c r="B10" s="17" t="inlineStr">
+        <is>
+          <t>Sist. Comun. CPF-COM-07</t>
+        </is>
+      </c>
+      <c r="C10" s="17" t="inlineStr">
+        <is>
+          <t>Gabinete comm Shelter 7; Stratix 5200/5800, SFPs, VLANs OT, patcheras FO</t>
+        </is>
+      </c>
+      <c r="D10" s="16" t="inlineStr">
+        <is>
+          <t>Hardware+Labor</t>
+        </is>
+      </c>
+      <c r="E10" s="18" t="inlineStr">
+        <is>
+          <t>CUBIERTO</t>
+        </is>
+      </c>
+      <c r="F10" s="17" t="inlineStr">
+        <is>
+          <t>D5F5E3</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="28" customHeight="1">
+      <c r="A11" s="16" t="inlineStr">
+        <is>
+          <t>3.1.1 #5</t>
+        </is>
+      </c>
+      <c r="B11" s="17" t="inlineStr">
+        <is>
+          <t>Sist. Comun. CPF-COM-SE3</t>
+        </is>
+      </c>
+      <c r="C11" s="17" t="inlineStr">
+        <is>
+          <t>Gabinete comm SE3 (shelter existente); patcheras FO y conversores re-incluidos (CT3 Q14)</t>
+        </is>
+      </c>
+      <c r="D11" s="16" t="inlineStr">
+        <is>
+          <t>Hardware+Labor</t>
+        </is>
+      </c>
+      <c r="E11" s="18" t="inlineStr">
+        <is>
+          <t>CUBIERTO</t>
+        </is>
+      </c>
+      <c r="F11" s="17" t="inlineStr">
+        <is>
+          <t>D5F5E3</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="28" customHeight="1">
+      <c r="A12" s="16" t="inlineStr">
+        <is>
+          <t>3.1.1 #6</t>
+        </is>
+      </c>
+      <c r="B12" s="17" t="inlineStr">
+        <is>
+          <t>Sist. Comun. CPF-COM-SE4</t>
+        </is>
+      </c>
+      <c r="C12" s="17" t="inlineStr">
+        <is>
+          <t>Gabinete comm SE4 (shelter existente); misma lógica que COM-SE3</t>
+        </is>
+      </c>
+      <c r="D12" s="16" t="inlineStr">
+        <is>
+          <t>Hardware+Labor</t>
+        </is>
+      </c>
+      <c r="E12" s="18" t="inlineStr">
+        <is>
+          <t>CUBIERTO</t>
+        </is>
+      </c>
+      <c r="F12" s="17" t="inlineStr">
+        <is>
+          <t>D5F5E3</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="28" customHeight="1">
+      <c r="A13" s="16" t="inlineStr">
+        <is>
+          <t>3.1.1 #7</t>
+        </is>
+      </c>
+      <c r="B13" s="17" t="inlineStr">
+        <is>
+          <t>Ingeniería Ctrl + Telesupervision</t>
+        </is>
+      </c>
+      <c r="C13" s="17" t="inlineStr">
+        <is>
+          <t>Todos los documentos de la lista XX-XXX-I-LD-CPF2-0.xlsx</t>
+        </is>
+      </c>
+      <c r="D13" s="16" t="inlineStr">
+        <is>
+          <t>Mano de Obra</t>
+        </is>
+      </c>
+      <c r="E13" s="18" t="inlineStr">
+        <is>
+          <t>CUBIERTO</t>
+        </is>
+      </c>
+      <c r="F13" s="17" t="inlineStr">
+        <is>
+          <t>D5F5E3</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="28" customHeight="1">
+      <c r="A14" s="16" t="inlineStr">
+        <is>
+          <t>3.1.1 #8</t>
+        </is>
+      </c>
+      <c r="B14" s="17" t="inlineStr">
+        <is>
+          <t>Config + FAT Ctrl Integral (PCS7,8,5,6,600)</t>
+        </is>
+      </c>
+      <c r="C14" s="17" t="inlineStr">
+        <is>
+          <t>Programación RTU ControlLogix; FAT eléctrica/lógica todos los gabinetes PCS</t>
+        </is>
+      </c>
+      <c r="D14" s="16" t="inlineStr">
+        <is>
+          <t>Mano de Obra</t>
+        </is>
+      </c>
+      <c r="E14" s="18" t="inlineStr">
+        <is>
+          <t>CUBIERTO</t>
+        </is>
+      </c>
+      <c r="F14" s="17" t="inlineStr">
+        <is>
+          <t>D5F5E3</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="28" customHeight="1">
+      <c r="A15" s="16" t="inlineStr">
+        <is>
+          <t>3.1.1 #9</t>
+        </is>
+      </c>
+      <c r="B15" s="17" t="inlineStr">
+        <is>
+          <t>Config + FAT SCADA (PCS+SIS: ESD6/7/8, PSS6/7/8, USS5/6, SS600)</t>
+        </is>
+      </c>
+      <c r="C15" s="17" t="inlineStr">
+        <is>
+          <t>Programación FactoryTalk; integración SCADA con sistemas HIMA. Requiere personal HIMA en FAT</t>
+        </is>
+      </c>
+      <c r="D15" s="16" t="inlineStr">
+        <is>
+          <t>Mano de Obra</t>
+        </is>
+      </c>
+      <c r="E15" s="18" t="inlineStr">
+        <is>
+          <t>CUBIERTO</t>
+        </is>
+      </c>
+      <c r="F15" s="17" t="inlineStr">
+        <is>
+          <t>D5F5E3</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="28" customHeight="1">
+      <c r="A16" s="16" t="inlineStr">
+        <is>
+          <t>3.1.1 #10</t>
+        </is>
+      </c>
+      <c r="B16" s="17" t="inlineStr">
+        <is>
+          <t>Config + FAT Sistema de Comunicaciones</t>
+        </is>
+      </c>
+      <c r="C16" s="17" t="inlineStr">
+        <is>
+          <t>Stratix, VLANs, Modbus TCP paquetizados (10 Skids A-H), Ethernet/IP, OPC</t>
+        </is>
+      </c>
+      <c r="D16" s="16" t="inlineStr">
+        <is>
+          <t>Mano de Obra</t>
+        </is>
+      </c>
+      <c r="E16" s="18" t="inlineStr">
+        <is>
+          <t>CUBIERTO</t>
+        </is>
+      </c>
+      <c r="F16" s="17" t="inlineStr">
+        <is>
+          <t>D5F5E3</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="28" customHeight="1">
+      <c r="A17" s="16" t="inlineStr">
+        <is>
+          <t>3.1.1 #11</t>
+        </is>
+      </c>
+      <c r="B17" s="17" t="inlineStr">
+        <is>
+          <t>Pruebas PMS BA (2 config. + viajes incl.)</t>
+        </is>
+      </c>
+      <c r="C17" s="17" t="inlineStr">
+        <is>
+          <t>Integración ABB 800xA en oficinas PP Buenos Aires; gastos cubiertos en precio cerrado</t>
+        </is>
+      </c>
+      <c r="D17" s="16" t="inlineStr">
+        <is>
+          <t>Mano de Obra</t>
+        </is>
+      </c>
+      <c r="E17" s="18" t="inlineStr">
+        <is>
+          <t>CUBIERTO</t>
+        </is>
+      </c>
+      <c r="F17" s="17" t="inlineStr">
+        <is>
+          <t>D5F5E3</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="28" customHeight="1">
+      <c r="A18" s="19" t="inlineStr">
+        <is>
+          <t>3.1.1 #12</t>
+        </is>
+      </c>
+      <c r="B18" s="20" t="inlineStr">
+        <is>
+          <t>Implementación Curva Bomba Flowserve en PLC+HMI</t>
+        </is>
+      </c>
+      <c r="C18" s="20" t="inlineStr">
+        <is>
+          <t>Era OPCIONAL en técnica. Ahora ítem cerrado. Requiere especificación de Pluspetrol.</t>
+        </is>
+      </c>
+      <c r="D18" s="19" t="inlineStr">
+        <is>
+          <t>Mano de Obra</t>
+        </is>
+      </c>
+      <c r="E18" s="21" t="inlineStr">
+        <is>
+          <t>NUEVO/OK</t>
+        </is>
+      </c>
+      <c r="F18" s="20" t="inlineStr">
+        <is>
+          <t>EBF5FB</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="28" customHeight="1">
+      <c r="A19" s="19" t="inlineStr">
+        <is>
+          <t>3.1.1 #13</t>
+        </is>
+      </c>
+      <c r="B19" s="20" t="inlineStr">
+        <is>
+          <t>Implementación Curva Bomba Flowserve en SCADA</t>
+        </is>
+      </c>
+      <c r="C19" s="20" t="inlineStr">
+        <is>
+          <t>Era OPCIONAL en técnica. Ahora ítem cerrado. Requiere especificación de Pluspetrol.</t>
+        </is>
+      </c>
+      <c r="D19" s="19" t="inlineStr">
+        <is>
+          <t>Mano de Obra</t>
+        </is>
+      </c>
+      <c r="E19" s="21" t="inlineStr">
+        <is>
+          <t>NUEVO/OK</t>
+        </is>
+      </c>
+      <c r="F19" s="20" t="inlineStr">
+        <is>
+          <t>EBF5FB</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="28" customHeight="1">
+      <c r="A20" s="16" t="inlineStr">
+        <is>
+          <t>3.1.2 #1</t>
+        </is>
+      </c>
+      <c r="B20" s="17" t="inlineStr">
+        <is>
+          <t>Repuestos Mínimos Recomendados PEM</t>
+        </is>
+      </c>
+      <c r="C20" s="17" t="inlineStr">
+        <is>
+          <t>Ítems de reemplazo rápido para equipos críticos (Sección 1.4 oferta técnica)</t>
+        </is>
+      </c>
+      <c r="D20" s="16" t="inlineStr">
+        <is>
+          <t>Repuestos</t>
+        </is>
+      </c>
+      <c r="E20" s="18" t="inlineStr">
+        <is>
+          <t>CUBIERTO</t>
+        </is>
+      </c>
+      <c r="F20" s="17" t="inlineStr">
+        <is>
+          <t>D5F5E3</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="28" customHeight="1">
+      <c r="A21" s="22" t="inlineStr">
+        <is>
+          <t>3.1.4 #1</t>
+        </is>
+      </c>
+      <c r="B21" s="23" t="inlineStr">
+        <is>
+          <t>Seguro Almacenaje ESD-SC-07/08 (mensual)</t>
+        </is>
+      </c>
+      <c r="C21" s="23" t="inlineStr">
+        <is>
+          <t>Equipo ya en Inauco. Factura desde Mayo 2026 — ANTES de OC. Negociar inicio desde OC.</t>
+        </is>
+      </c>
+      <c r="D21" s="22" t="inlineStr">
+        <is>
+          <t>Seguros</t>
+        </is>
+      </c>
+      <c r="E21" s="24" t="inlineStr">
+        <is>
+          <t>ATENCIÓN</t>
+        </is>
+      </c>
+      <c r="F21" s="23" t="inlineStr">
+        <is>
+          <t>FDEBD0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="28" customHeight="1">
+      <c r="A22" s="16" t="inlineStr">
+        <is>
+          <t>3.1.4 #2</t>
+        </is>
+      </c>
+      <c r="B22" s="17" t="inlineStr">
+        <is>
+          <t>Seguro Almacenaje PSS-007A/B + FGS/ESD-007</t>
+        </is>
+      </c>
+      <c r="C22" s="17" t="inlineStr">
+        <is>
+          <t>Desde OC hasta entrega en yacimiento. Normal.</t>
+        </is>
+      </c>
+      <c r="D22" s="16" t="inlineStr">
+        <is>
+          <t>Seguros</t>
+        </is>
+      </c>
+      <c r="E22" s="18" t="inlineStr">
+        <is>
+          <t>CUBIERTO</t>
+        </is>
+      </c>
+      <c r="F22" s="17" t="inlineStr">
+        <is>
+          <t>D5F5E3</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="28" customHeight="1">
+      <c r="A23" s="25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B23" s="26" t="inlineStr">
+        <is>
+          <t>PEM / Asistencia Startup</t>
+        </is>
+      </c>
+      <c r="C23" s="26" t="inlineStr">
+        <is>
+          <t>Mencionada en técnica como A Demanda pero SIN estimación de días en comercial</t>
+        </is>
+      </c>
+      <c r="D23" s="25" t="inlineStr">
+        <is>
+          <t>A Demanda</t>
+        </is>
+      </c>
+      <c r="E23" s="27" t="inlineStr">
+        <is>
+          <t>BRECHA</t>
+        </is>
+      </c>
+      <c r="F23" s="26" t="inlineStr">
+        <is>
+          <t>FADBD8</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="28" customHeight="1">
+      <c r="A24" s="25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B24" s="26" t="inlineStr">
+        <is>
+          <t>Pre-comisionado señales I/O (&gt;80% req.)</t>
+        </is>
+      </c>
+      <c r="C24" s="26" t="inlineStr">
+        <is>
+          <t>Condición para inicio de SAT. Sin estimación de jornadas ni asignación de responsabilidad</t>
+        </is>
+      </c>
+      <c r="D24" s="25" t="inlineStr">
+        <is>
+          <t>A Demanda</t>
+        </is>
+      </c>
+      <c r="E24" s="27" t="inlineStr">
+        <is>
+          <t>BRECHA</t>
+        </is>
+      </c>
+      <c r="F24" s="26" t="inlineStr">
+        <is>
+          <t>FADBD8</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="16" customHeight="1">
+      <c r="A26" s="28" t="inlineStr">
+        <is>
+          <t>2. JORNADAS A DEMANDA — SUGERENCIAS SECCIÓN 2 (NO LIMITATIVAS)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="16" customHeight="1">
+      <c r="A27" s="29" t="inlineStr">
+        <is>
+          <t>⚠ ALERTA: Días/Hombre de campo = 0 (CERO) en precio fijo. Todo SAT/comisionado/PEM es A Demanda sin cap contractual.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="20" customHeight="1">
+      <c r="A28" s="30" t="inlineStr">
+        <is>
+          <t>Actividad</t>
+        </is>
+      </c>
+      <c r="B28" s="30" t="inlineStr">
+        <is>
+          <t>Perfil / Ítem Ec.</t>
+        </is>
+      </c>
+      <c r="C28" s="30" t="inlineStr">
+        <is>
+          <t>Jornadas (días 8h)</t>
+        </is>
+      </c>
+      <c r="D28" s="30" t="inlineStr">
+        <is>
+          <t>Personas</t>
+        </is>
+      </c>
+      <c r="E28" s="30" t="inlineStr">
+        <is>
+          <t>Movilidad (#11)</t>
+        </is>
+      </c>
+      <c r="F28" s="30" t="inlineStr">
+        <is>
+          <t>Alojamiento (#12/noche)</t>
+        </is>
+      </c>
+      <c r="G28" s="30" t="inlineStr">
+        <is>
+          <t>Observación</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="28" customHeight="1">
+      <c r="A29" s="23" t="inlineStr">
+        <is>
+          <t>Reloc. Controladores Shelter 6 → Remota 7B</t>
+        </is>
+      </c>
+      <c r="B29" s="23" t="inlineStr">
+        <is>
+          <t>Configurador (Ítem 1)
+Conexionista (Ítem 7)</t>
+        </is>
+      </c>
+      <c r="C29" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="D29" s="22" t="inlineStr">
+        <is>
+          <t>1+1</t>
+        </is>
+      </c>
+      <c r="E29" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="F29" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="G29" s="23" t="inlineStr">
+        <is>
+          <t>BAJO — probablemente insuficiente para relocalizar ControlLogix + reconfig PRP + ensayo</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="28" customHeight="1">
+      <c r="A30" s="31" t="inlineStr">
+        <is>
+          <t>Vínculos Ethernet PCS → COM (tendido + certificación)</t>
+        </is>
+      </c>
+      <c r="B30" s="31" t="inlineStr">
+        <is>
+          <t>Conexionista (Ítem 7)</t>
+        </is>
+      </c>
+      <c r="C30" s="32" t="n">
+        <v>15</v>
+      </c>
+      <c r="D30" s="32" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E30" s="32" t="n"/>
+      <c r="F30" s="32" t="n">
+        <v>13</v>
+      </c>
+      <c r="G30" s="31" t="inlineStr">
+        <is>
+          <t>Razonable para tramos físicos entre shelters</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="28" customHeight="1">
+      <c r="A31" s="31" t="inlineStr">
+        <is>
+          <t>SAT + Comisionado PCS (07a + 07b)</t>
+        </is>
+      </c>
+      <c r="B31" s="31" t="inlineStr">
+        <is>
+          <t>Configurador (Ítem 1)
+Conexionista (Ítem 7)</t>
+        </is>
+      </c>
+      <c r="C31" s="32" t="n">
+        <v>55</v>
+      </c>
+      <c r="D31" s="32" t="inlineStr">
+        <is>
+          <t>1+1</t>
+        </is>
+      </c>
+      <c r="E31" s="32" t="n">
+        <v>55</v>
+      </c>
+      <c r="F31" s="32" t="n">
+        <v>108</v>
+      </c>
+      <c r="G31" s="31" t="inlineStr">
+        <is>
+          <t>Crítico. ~10 señales/día en cond. ideales. Depende I/O precomisionado &gt;80%</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="28" customHeight="1">
+      <c r="A32" s="31" t="inlineStr">
+        <is>
+          <t>SAT + Comisionado SCADA PCS (FactoryTalk)</t>
+        </is>
+      </c>
+      <c r="B32" s="31" t="inlineStr">
+        <is>
+          <t>Configurador (Ítem 1)
+QAQC (Ítem 6)</t>
+        </is>
+      </c>
+      <c r="C32" s="32" t="n">
+        <v>65</v>
+      </c>
+      <c r="D32" s="32" t="inlineStr">
+        <is>
+          <t>1+1</t>
+        </is>
+      </c>
+      <c r="E32" s="32" t="n">
+        <v>65</v>
+      </c>
+      <c r="F32" s="32" t="n">
+        <v>128</v>
+      </c>
+      <c r="G32" s="31" t="inlineStr">
+        <is>
+          <t>Incluye PCS5, PCS6, PCS600 existentes ampliados. Razonable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="28" customHeight="1">
+      <c r="A33" s="23" t="inlineStr">
+        <is>
+          <t>SAT + Comisionado SCADA SIS (ESD/F&amp;G/PSS/USS)</t>
+        </is>
+      </c>
+      <c r="B33" s="23" t="inlineStr">
+        <is>
+          <t>Configurador (Ítem 1)
+QAQC (Ítem 6)</t>
+        </is>
+      </c>
+      <c r="C33" s="22" t="n">
+        <v>100</v>
+      </c>
+      <c r="D33" s="22" t="inlineStr">
+        <is>
+          <t>1+1</t>
+        </is>
+      </c>
+      <c r="E33" s="22" t="n">
+        <v>100</v>
+      </c>
+      <c r="F33" s="22" t="n">
+        <v>198</v>
+      </c>
+      <c r="G33" s="23" t="inlineStr">
+        <is>
+          <t>ALTO. Requiere presencia personal HIMA en campo. Validar disponibilidad.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="28" customHeight="1">
+      <c r="A34" s="31" t="inlineStr">
+        <is>
+          <t>Prueba Matriz C&amp;E SCADA</t>
+        </is>
+      </c>
+      <c r="B34" s="31" t="inlineStr">
+        <is>
+          <t>Configurador (Ítem 1)</t>
+        </is>
+      </c>
+      <c r="C34" s="32" t="n">
+        <v>15</v>
+      </c>
+      <c r="D34" s="32" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E34" s="32" t="n">
+        <v>15</v>
+      </c>
+      <c r="F34" s="32" t="n">
+        <v>14</v>
+      </c>
+      <c r="G34" s="31" t="inlineStr">
+        <is>
+          <t>Última etapa de validación. Requiere personal SIS presente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="28" customHeight="1">
+      <c r="A35" s="26" t="inlineStr">
+        <is>
+          <t>Puesta en Marcha (PEM) — Startup</t>
+        </is>
+      </c>
+      <c r="B35" s="26" t="inlineStr">
+        <is>
+          <t>Configurador (Ítem 1 ó 2)</t>
+        </is>
+      </c>
+      <c r="C35" s="27" t="inlineStr">
+        <is>
+          <t>NO ESTIMADO</t>
+        </is>
+      </c>
+      <c r="D35" s="25" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="E35" s="25" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="F35" s="25" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="G35" s="26" t="inlineStr">
+        <is>
+          <t>BRECHA — no hay estimación. Fase separada del comisionado en arranque real.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="28" customHeight="1">
+      <c r="A36" s="26" t="inlineStr">
+        <is>
+          <t>Pre-comisionado señales I/O (&gt;80% para habilitar SAT)</t>
+        </is>
+      </c>
+      <c r="B36" s="26" t="inlineStr">
+        <is>
+          <t>Cuadrilla 2 (Ítem 9) ó Conexionista (Ítem 7)</t>
+        </is>
+      </c>
+      <c r="C36" s="27" t="inlineStr">
+        <is>
+          <t>NO ESTIMADO</t>
+        </is>
+      </c>
+      <c r="D36" s="25" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="E36" s="25" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="F36" s="25" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="G36" s="26" t="inlineStr">
+        <is>
+          <t>BRECHA — condición previa a SAT sin días asignados. Responsabilidad a definir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="18" customHeight="1">
+      <c r="A37" s="33" t="inlineStr">
+        <is>
+          <t>TOTALES SUGERIDOS (sin PEM ni precomisionado)</t>
+        </is>
+      </c>
+      <c r="B37" s="33" t="inlineStr"/>
+      <c r="C37" s="34" t="n">
+        <v>237</v>
+      </c>
+      <c r="D37" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E37" s="34" t="n">
+        <v>237</v>
+      </c>
+      <c r="F37" s="34" t="n">
+        <v>463</v>
+      </c>
+      <c r="G37" s="34" t="inlineStr">
+        <is>
+          <t>~474 jornadas-persona totales (config+conexionista+QC)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="16" customHeight="1">
+      <c r="A39" s="35" t="inlineStr">
+        <is>
+          <t>3. CONDICIONES PARA ADJUDICACIÓN</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="20" customHeight="1">
+      <c r="A40" s="36" t="inlineStr">
+        <is>
+          <t>Cond.</t>
+        </is>
+      </c>
+      <c r="B40" s="36" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="C40" s="36" t="inlineStr">
+        <is>
+          <t>Título</t>
+        </is>
+      </c>
+      <c r="D40" s="36" t="inlineStr">
+        <is>
+          <t>Descripción resumida</t>
+        </is>
+      </c>
+      <c r="E40" s="36" t="inlineStr">
+        <is>
+          <t>Fecha Límite</t>
+        </is>
+      </c>
+      <c r="F40" s="36" t="inlineStr">
+        <is>
+          <t>Responsable</t>
+        </is>
+      </c>
+      <c r="G40" s="36" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="40" customHeight="1">
+      <c r="A41" s="25" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="B41" s="27" t="inlineStr">
+        <is>
+          <t>OBLIGATORIA</t>
+        </is>
+      </c>
+      <c r="C41" s="26" t="inlineStr">
+        <is>
+          <t>Caps Jornadas A Demanda</t>
+        </is>
+      </c>
+      <c r="D41" s="26" t="inlineStr">
+        <is>
+          <t>Anexar como condición contractual los topes máximos de jornadas (Sección 2 como límite +20%). SAT PCS: 110 p/días · SCADA PCS: 130 p/días · SCADA SIS: 200 p/días · C&amp;E: 15 días.</t>
+        </is>
+      </c>
+      <c r="E41" s="25" t="inlineStr">
+        <is>
+          <t>≤15/06/2026</t>
+        </is>
+      </c>
+      <c r="F41" s="25" t="inlineStr">
+        <is>
+          <t>PM + Contratos</t>
+        </is>
+      </c>
+      <c r="G41" s="37" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="40" customHeight="1">
+      <c r="A42" s="25" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+      <c r="B42" s="27" t="inlineStr">
+        <is>
+          <t>OBLIGATORIA</t>
+        </is>
+      </c>
+      <c r="C42" s="26" t="inlineStr">
+        <is>
+          <t>Estimación PEM y Pre-comisionado</t>
+        </is>
+      </c>
+      <c r="D42" s="26" t="inlineStr">
+        <is>
+          <t>Solicitar a Inauco estimación de jornadas para PEM/startup y precomisionado I/O. Ítems 7 y 9 del catálogo A Demanda son las herramientas correctas.</t>
+        </is>
+      </c>
+      <c r="E42" s="25" t="inlineStr">
+        <is>
+          <t>≤15/06/2026</t>
+        </is>
+      </c>
+      <c r="F42" s="25" t="inlineStr">
+        <is>
+          <t>Inauco → PM</t>
+        </is>
+      </c>
+      <c r="G42" s="37" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="40" customHeight="1">
+      <c r="A43" s="25" t="inlineStr">
+        <is>
+          <t>C3</t>
+        </is>
+      </c>
+      <c r="B43" s="27" t="inlineStr">
+        <is>
+          <t>OBLIGATORIA</t>
+        </is>
+      </c>
+      <c r="C43" s="26" t="inlineStr">
+        <is>
+          <t>Inicio Seguro Almacenaje desde OC</t>
+        </is>
+      </c>
+      <c r="D43" s="26" t="inlineStr">
+        <is>
+          <t>Negociar que Ítem 3.1.4.1 (ESD-SC-07/08) facture desde OC, no retroactivo desde Mayo 2026.</t>
+        </is>
+      </c>
+      <c r="E43" s="25" t="inlineStr">
+        <is>
+          <t>≤15/06/2026</t>
+        </is>
+      </c>
+      <c r="F43" s="25" t="inlineStr">
+        <is>
+          <t>PM + Adm.</t>
+        </is>
+      </c>
+      <c r="G43" s="37" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="40" customHeight="1">
+      <c r="A44" s="22" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="B44" s="24" t="inlineStr">
+        <is>
+          <t>RECOMENDADA</t>
+        </is>
+      </c>
+      <c r="C44" s="23" t="inlineStr">
+        <is>
+          <t>Revisión Relocalización Shelf 6</t>
+        </is>
+      </c>
+      <c r="D44" s="23" t="inlineStr">
+        <is>
+          <t>Exigir desglose detallado para relocalización ControlLogix Shelter 6 → Remota 7B. 2 días claramente insuficiente para reconexión, reconfig PRP y ensayo.</t>
+        </is>
+      </c>
+      <c r="E44" s="22" t="inlineStr">
+        <is>
+          <t>≤20/06/2026</t>
+        </is>
+      </c>
+      <c r="F44" s="22" t="inlineStr">
+        <is>
+          <t>PM + Inauco</t>
+        </is>
+      </c>
+      <c r="G44" s="24" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="40" customHeight="1">
+      <c r="A45" s="22" t="inlineStr">
+        <is>
+          <t>C5</t>
+        </is>
+      </c>
+      <c r="B45" s="24" t="inlineStr">
+        <is>
+          <t>RECOMENDADA</t>
+        </is>
+      </c>
+      <c r="C45" s="23" t="inlineStr">
+        <is>
+          <t>Confirmar Perfil SCADA SAT (Ítem 1 vs. 2)</t>
+        </is>
+      </c>
+      <c r="D45" s="23" t="inlineStr">
+        <is>
+          <t>Verificar si comisionado SCADA SIS/PCS usa Ítem 1 (Control) o Ítem 2 (Telesupervision). Diferente tarifa, diferente perfil técnico.</t>
+        </is>
+      </c>
+      <c r="E45" s="22" t="inlineStr">
+        <is>
+          <t>≤20/06/2026</t>
+        </is>
+      </c>
+      <c r="F45" s="22" t="inlineStr">
+        <is>
+          <t>PM + Inauco</t>
+        </is>
+      </c>
+      <c r="G45" s="24" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="40" customHeight="1">
+      <c r="A46" s="22" t="inlineStr">
+        <is>
+          <t>C6</t>
+        </is>
+      </c>
+      <c r="B46" s="24" t="inlineStr">
+        <is>
+          <t>RECOMENDADA</t>
+        </is>
+      </c>
+      <c r="C46" s="23" t="inlineStr">
+        <is>
+          <t>Contingencia Jornadas No Hábiles</t>
+        </is>
+      </c>
+      <c r="D46" s="23" t="inlineStr">
+        <is>
+          <t>Presupuestar reserva 15-20% sobre jornadas estimadas para sábados/domingos/feriados (certificados al 100% adicional según oferta).</t>
+        </is>
+      </c>
+      <c r="E46" s="22" t="inlineStr">
+        <is>
+          <t>Antes OC</t>
+        </is>
+      </c>
+      <c r="F46" s="22" t="inlineStr">
+        <is>
+          <t>PM + Finanzas</t>
+        </is>
+      </c>
+      <c r="G46" s="24" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="40" customHeight="1">
+      <c r="A47" s="19" t="inlineStr">
+        <is>
+          <t>C7</t>
+        </is>
+      </c>
+      <c r="B47" s="21" t="inlineStr">
+        <is>
+          <t>INFORMATIVA</t>
+        </is>
+      </c>
+      <c r="C47" s="20" t="inlineStr">
+        <is>
+          <t>Verificar Especif. Flowserve</t>
+        </is>
+      </c>
+      <c r="D47" s="20" t="inlineStr">
+        <is>
+          <t>Confirmar que Pluspetrol/AESA proveen la especificación de curvas de bomba Flowserve para que Inauco pueda ejecutar Ítems 12 y 13.</t>
+        </is>
+      </c>
+      <c r="E47" s="19" t="inlineStr">
+        <is>
+          <t>≤30/09/2026</t>
+        </is>
+      </c>
+      <c r="F47" s="19" t="inlineStr">
+        <is>
+          <t>AESA → PM</t>
+        </is>
+      </c>
+      <c r="G47" s="38" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="16" customHeight="1">
+      <c r="A49" s="14" t="inlineStr">
+        <is>
+          <t>4. CONDICIONES DE PAGO</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="18" customHeight="1">
+      <c r="A50" s="15" t="inlineStr">
+        <is>
+          <t>Concepto</t>
+        </is>
+      </c>
+      <c r="B50" s="15" t="inlineStr">
+        <is>
+          <t>Condición</t>
+        </is>
+      </c>
+      <c r="C50" s="15" t="inlineStr">
+        <is>
+          <t>Momento estimado</t>
+        </is>
+      </c>
+      <c r="D50" s="15" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E50" s="15" t="inlineStr">
+        <is>
+          <t>Modalidad</t>
+        </is>
+      </c>
+      <c r="F50" s="15" t="inlineStr">
+        <is>
+          <t>Observación</t>
+        </is>
+      </c>
+      <c r="G50" s="15" t="inlineStr"/>
+    </row>
+    <row r="51" ht="22" customHeight="1">
+      <c r="A51" s="31" t="inlineStr">
+        <is>
+          <t>Hardware Ítems 1-6 + Rep. (75%)</t>
+        </is>
+      </c>
+      <c r="B51" s="31" t="inlineStr">
+        <is>
+          <t>Recepción materiales críticos</t>
+        </is>
+      </c>
+      <c r="C51" s="32" t="inlineStr">
+        <is>
+          <t>~Ago-Sep 2026</t>
+        </is>
+      </c>
+      <c r="D51" s="32" t="inlineStr">
+        <is>
+          <t>75%</t>
+        </is>
+      </c>
+      <c r="E51" s="32" t="inlineStr">
+        <is>
+          <t>Remito proveedor</t>
+        </is>
+      </c>
+      <c r="F51" s="31" t="inlineStr">
+        <is>
+          <t>Pago mayor al inicio. Prever flujo de caja.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="22" customHeight="1">
+      <c r="A52" s="39" t="inlineStr">
+        <is>
+          <t>Hardware 25% restante</t>
+        </is>
+      </c>
+      <c r="B52" s="39" t="inlineStr">
+        <is>
+          <t>Contra FAT Ítems 1-6</t>
+        </is>
+      </c>
+      <c r="C52" s="40" t="inlineStr">
+        <is>
+          <t>Feb 2027 (FAT)</t>
+        </is>
+      </c>
+      <c r="D52" s="40" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="E52" s="40" t="inlineStr">
+        <is>
+          <t>Remito FAT</t>
+        </is>
+      </c>
+      <c r="F52" s="39" t="inlineStr">
+        <is>
+          <t>Pequeño desembolso post-FAT</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="22" customHeight="1">
+      <c r="A53" s="31" t="inlineStr">
+        <is>
+          <t>M.O. Ingeniería/Config/FAT (Ítems 7-10): 20% adelanto</t>
+        </is>
+      </c>
+      <c r="B53" s="31" t="inlineStr">
+        <is>
+          <t>Con OC</t>
+        </is>
+      </c>
+      <c r="C53" s="32" t="inlineStr">
+        <is>
+          <t>Jun-Jul 2026</t>
+        </is>
+      </c>
+      <c r="D53" s="32" t="inlineStr">
+        <is>
+          <t>20%</t>
+        </is>
+      </c>
+      <c r="E53" s="32" t="inlineStr">
+        <is>
+          <t>Anticipo con OC</t>
+        </is>
+      </c>
+      <c r="F53" s="31" t="inlineStr">
+        <is>
+          <t>Para iniciar ingeniería</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="22" customHeight="1">
+      <c r="A54" s="39" t="inlineStr">
+        <is>
+          <t>M.O. 80% restante</t>
+        </is>
+      </c>
+      <c r="B54" s="39" t="inlineStr">
+        <is>
+          <t>Certificaciones mensuales / avance</t>
+        </is>
+      </c>
+      <c r="C54" s="40" t="inlineStr">
+        <is>
+          <t>Durante obra (30 DFF)</t>
+        </is>
+      </c>
+      <c r="D54" s="40" t="inlineStr">
+        <is>
+          <t>80%</t>
+        </is>
+      </c>
+      <c r="E54" s="40" t="inlineStr">
+        <is>
+          <t>Certificaciones mensuales</t>
+        </is>
+      </c>
+      <c r="F54" s="39" t="inlineStr">
+        <is>
+          <t>Sistema de certificaciones requerido</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="22" customHeight="1">
+      <c r="A55" s="31" t="inlineStr">
+        <is>
+          <t>PMS Buenos Aires (Ítem 11)</t>
+        </is>
+      </c>
+      <c r="B55" s="31" t="inlineStr">
+        <is>
+          <t>Certificación pruebas BA</t>
+        </is>
+      </c>
+      <c r="C55" s="32" t="inlineStr">
+        <is>
+          <t>Post-ensayos BA</t>
+        </is>
+      </c>
+      <c r="D55" s="32" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="E55" s="32" t="inlineStr">
+        <is>
+          <t>Certificación prueba</t>
+        </is>
+      </c>
+      <c r="F55" s="31" t="inlineStr">
+        <is>
+          <t>Pago único al completar BA</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="22" customHeight="1">
+      <c r="A56" s="39" t="inlineStr">
+        <is>
+          <t>A Demanda (Ítem 3.1.3)</t>
+        </is>
+      </c>
+      <c r="B56" s="39" t="inlineStr">
+        <is>
+          <t>Remito firmado por inspección</t>
+        </is>
+      </c>
+      <c r="C56" s="40" t="inlineStr">
+        <is>
+          <t>Por jornada (30 DFF)</t>
+        </is>
+      </c>
+      <c r="D56" s="40" t="inlineStr">
+        <is>
+          <t>Unit.</t>
+        </is>
+      </c>
+      <c r="E56" s="40" t="inlineStr">
+        <is>
+          <t>Por jornada</t>
+        </is>
+      </c>
+      <c r="F56" s="39" t="inlineStr">
+        <is>
+          <t>Seguimiento estricto de remitos</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="22" customHeight="1">
+      <c r="A57" s="23" t="inlineStr">
+        <is>
+          <t>Seguro ESD-SC-07/08 (3.1.4.1)</t>
+        </is>
+      </c>
+      <c r="B57" s="23" t="inlineStr">
+        <is>
+          <t>Mensual desde Mayo 2026</t>
+        </is>
+      </c>
+      <c r="C57" s="22" t="inlineStr">
+        <is>
+          <t>RETROACTIVO — negociar</t>
+        </is>
+      </c>
+      <c r="D57" s="22" t="inlineStr">
+        <is>
+          <t>Mensual</t>
+        </is>
+      </c>
+      <c r="E57" s="22" t="inlineStr">
+        <is>
+          <t>Mensual desde OC (negociar)</t>
+        </is>
+      </c>
+      <c r="F57" s="23" t="inlineStr">
+        <is>
+          <t>Gap G5 — riesgo retroactivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="22" customHeight="1">
+      <c r="A58" s="39" t="inlineStr">
+        <is>
+          <t>Seguro PSS+FGS (3.1.4.2)</t>
+        </is>
+      </c>
+      <c r="B58" s="39" t="inlineStr">
+        <is>
+          <t>Mensual desde OC</t>
+        </is>
+      </c>
+      <c r="C58" s="40" t="inlineStr">
+        <is>
+          <t>Mensual</t>
+        </is>
+      </c>
+      <c r="D58" s="40" t="inlineStr">
+        <is>
+          <t>Mensual</t>
+        </is>
+      </c>
+      <c r="E58" s="40" t="inlineStr">
+        <is>
+          <t>Mensual desde OC</t>
+        </is>
+      </c>
+      <c r="F58" s="39" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="16" customHeight="1">
+      <c r="A60" s="14" t="inlineStr">
+        <is>
+          <t>5. PRÓXIMOS PASOS — RUTA CRÍTICA ADJUDICACIÓN</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="18" customHeight="1">
+      <c r="A61" s="15" t="inlineStr">
+        <is>
+          <t>Fecha Límite</t>
+        </is>
+      </c>
+      <c r="B61" s="15" t="inlineStr">
+        <is>
+          <t>Actividad</t>
+        </is>
+      </c>
+      <c r="C61" s="15" t="inlineStr">
+        <is>
+          <t>Detalle</t>
+        </is>
+      </c>
+      <c r="D61" s="15" t="inlineStr">
+        <is>
+          <t>Responsable</t>
+        </is>
+      </c>
+      <c r="E61" s="15" t="inlineStr">
+        <is>
+          <t>Prioridad</t>
+        </is>
+      </c>
+      <c r="F61" s="15" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+      <c r="G61" s="15" t="inlineStr"/>
+    </row>
+    <row r="62" ht="22" customHeight="1">
+      <c r="A62" s="25" t="inlineStr">
+        <is>
+          <t>Inmediato</t>
+        </is>
+      </c>
+      <c r="B62" s="26" t="inlineStr">
+        <is>
+          <t>Enviar condiciones C1-C3 a Inauco</t>
+        </is>
+      </c>
+      <c r="C62" s="26" t="inlineStr">
+        <is>
+          <t>Plazo respuesta 5 días hábiles</t>
+        </is>
+      </c>
+      <c r="D62" s="25" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="E62" s="27" t="inlineStr">
+        <is>
+          <t>CRÍTICA</t>
+        </is>
+      </c>
+      <c r="F62" s="37" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="22" customHeight="1">
+      <c r="A63" s="25" t="inlineStr">
+        <is>
+          <t>≤15/06/2026</t>
+        </is>
+      </c>
+      <c r="B63" s="26" t="inlineStr">
+        <is>
+          <t>Acordar caps jornadas + inicio seguro</t>
+        </is>
+      </c>
+      <c r="C63" s="26" t="inlineStr">
+        <is>
+          <t>Negociar Anexo A Demanda caps y fecha seguro ESD desde OC</t>
+        </is>
+      </c>
+      <c r="D63" s="25" t="inlineStr">
+        <is>
+          <t>PM + Contratos</t>
+        </is>
+      </c>
+      <c r="E63" s="27" t="inlineStr">
+        <is>
+          <t>CRÍTICA</t>
+        </is>
+      </c>
+      <c r="F63" s="37" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="22" customHeight="1">
+      <c r="A64" s="22" t="inlineStr">
+        <is>
+          <t>≤20/06/2026</t>
+        </is>
+      </c>
+      <c r="B64" s="23" t="inlineStr">
+        <is>
+          <t>Obtener estimación PEM y precomisionado</t>
+        </is>
+      </c>
+      <c r="C64" s="23" t="inlineStr">
+        <is>
+          <t>Confirmar perfil Ítem 1 vs. 2 para SCADA SAT</t>
+        </is>
+      </c>
+      <c r="D64" s="22" t="inlineStr">
+        <is>
+          <t>PM + Inauco</t>
+        </is>
+      </c>
+      <c r="E64" s="24" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="F64" s="24" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="22" customHeight="1">
+      <c r="A65" s="25" t="inlineStr">
+        <is>
+          <t>≤28/07/2026</t>
+        </is>
+      </c>
+      <c r="B65" s="26" t="inlineStr">
+        <is>
+          <t>Emitir Orden de Compra</t>
+        </is>
+      </c>
+      <c r="C65" s="26" t="inlineStr">
+        <is>
+          <t>Fecha límite validez oferta (60 días desde 29/05/2026)</t>
+        </is>
+      </c>
+      <c r="D65" s="25" t="inlineStr">
+        <is>
+          <t>Compras/PM</t>
+        </is>
+      </c>
+      <c r="E65" s="27" t="inlineStr">
+        <is>
+          <t>CRÍTICA</t>
+        </is>
+      </c>
+      <c r="F65" s="37" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="22" customHeight="1">
+      <c r="A66" s="25" t="inlineStr">
+        <is>
+          <t>01/07/2026</t>
+        </is>
+      </c>
+      <c r="B66" s="26" t="inlineStr">
+        <is>
+          <t>Confirmar entrega HIMA</t>
+        </is>
+      </c>
+      <c r="C66" s="26" t="inlineStr">
+        <is>
+          <t>Sin buffer en path crítico. Inauco necesita HIMA para FAT integral.</t>
+        </is>
+      </c>
+      <c r="D66" s="25" t="inlineStr">
+        <is>
+          <t>PM + HIMA/AESA</t>
+        </is>
+      </c>
+      <c r="E66" s="27" t="inlineStr">
+        <is>
+          <t>CRÍTICA</t>
+        </is>
+      </c>
+      <c r="F66" s="37" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="22" customHeight="1">
+      <c r="A67" s="22" t="inlineStr">
+        <is>
+          <t>≤30/09/2026</t>
+        </is>
+      </c>
+      <c r="B67" s="23" t="inlineStr">
+        <is>
+          <t>Entregar documentación freezing point</t>
+        </is>
+      </c>
+      <c r="C67" s="23" t="inlineStr">
+        <is>
+          <t>Listado señales + P&amp;ID + MCE + Arq. General — 16 sem antes FAT 27/01/2027</t>
+        </is>
+      </c>
+      <c r="D67" s="22" t="inlineStr">
+        <is>
+          <t>AESA → Inauco</t>
+        </is>
+      </c>
+      <c r="E67" s="24" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="F67" s="24" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="22" customHeight="1">
+      <c r="A68" s="19" t="inlineStr">
+        <is>
+          <t>≤30/09/2026</t>
+        </is>
+      </c>
+      <c r="B68" s="20" t="inlineStr">
+        <is>
+          <t>Verificar especif. Flowserve</t>
+        </is>
+      </c>
+      <c r="C68" s="20" t="inlineStr">
+        <is>
+          <t>Pluspetrol/AESA entregan especificación curvas bomba para Ítems 12/13</t>
+        </is>
+      </c>
+      <c r="D68" s="19" t="inlineStr">
+        <is>
+          <t>AESA</t>
+        </is>
+      </c>
+      <c r="E68" s="21" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="F68" s="38" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="10">
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A27:G27"/>
+    <mergeCell ref="A3:G3"/>
+    <mergeCell ref="A39:G39"/>
+    <mergeCell ref="A26:G26"/>
+    <mergeCell ref="E6"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A60:G60"/>
+    <mergeCell ref="A49:G49"/>
+    <mergeCell ref="A5:G5"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -681,7 +2774,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1518,7 +3611,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2067,7 +4160,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2761,7 +4854,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3420,7 +5513,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3853,7 +5946,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>